<commit_message>
docs: clarify the hook — one game, one theme; variety lives inside it
The visual-variety hook means many distinct tilesets/characters/monsters
within the single world the designer picks in design/ — not a
theme-swapping mechanic. The archived space reskin was a pipeline
experiment, not a direction. Clarified in CLAUDE.md, archive/README.md,
and the workbook's Art & Tilesets tab.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NaK47EKCSGuPn6dcCqQ5r9
</commit_message>
<xml_diff>
--- a/design/game-bible.xlsx
+++ b/design/game-bible.xlsx
@@ -569,7 +569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C32"/>
+  <dimension ref="B2:C32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -577,7 +577,6 @@
     <col width="88" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="38" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -592,7 +591,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -660,7 +658,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="B12" s="3" t="inlineStr">
         <is>
@@ -1812,10 +1809,11 @@
     <row r="2">
       <c r="A2" s="17" t="inlineStr">
         <is>
-          <t>The visual-variety hook made concrete: the themed art sets the cartridge swaps between. One row per set — where it's used, its palette mood, its key tiles. Hard limit: any 16×16 block gets 3 colors + the shared backdrop (see framework/ASSETS.md).</t>
-        </is>
-      </c>
-    </row>
+          <t>The look of the game's ONE world, organized into themed art sets — one row per set: where it's used, its palette mood, its key tiles. Variety means each region/town/dungeon of the single chosen theme looks distinct (this is not a theme-swap mechanic). Hard limit: any 16×16 block gets 3 colors + the shared backdrop (see framework/ASSETS.md).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
         <is>
@@ -2075,10 +2073,11 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="18" t="inlineStr">
         <is>
-          <t>Variety comes from themed SETS the cartridge swaps per area/scene — design in sets, not one-off art everywhere. Placeholder rows sketch a DQ1-scale lineup; replace with our own.</t>
+          <t>Sets are how the hardware organizes one world's art (each area points at its own tile bank) — design in themed sets, not one-off art everywhere. Placeholder rows sketch a DQ1-scale lineup; replace them with sets from the chosen creative direction.</t>
         </is>
       </c>
     </row>
@@ -6255,7 +6254,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="9" t="inlineStr">
         <is>
@@ -7252,7 +7250,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="12" t="inlineStr">
         <is>

</xml_diff>